<commit_message>
Ambiguity calculations for narrow framing
</commit_message>
<xml_diff>
--- a/1_Data/RawData/PriceData/Düngemittelabfrage Altdaten - KAB - ab 2007 bis August 2021.xlsx
+++ b/1_Data/RawData/PriceData/Düngemittelabfrage Altdaten - KAB - ab 2007 bis August 2021.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wageningenur4-my.sharepoint.com/personal/riccardo_spada_wur_nl/Documents/Publication_2/1_Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wageningenur4-my.sharepoint.com/personal/riccardo_spada_wur_nl/Documents/publication_2/1_Data/RawData/PriceData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{4372643C-6710-415F-BA51-BAF8E95B67EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7A12900-4FC8-42B9-AB59-657C5ACA5A97}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{4372643C-6710-415F-BA51-BAF8E95B67EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A1A01A36-43D1-4F52-9DE6-0BF2968188B2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="28800" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KAS ab März 2007" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,20 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'SSA ab August 2009'!$A$3:$E$293</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TSP ab März 2007'!$A$3:$E$329</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>